<commit_message>
Day 3 send: 2 real emails (0 Indonesia, 2 Singapore)
Both country pools hit real exhaustion today, not just a slow batch:
Indonesia's day-3 research pass ran ~3x normal search volume (47
queries) and found zero new domain-matched-email prospects (one
contact-form-only lead, Nusantara Data Center, no verified email);
Singapore found only 2 clean rows after 3 prior batches already covered
most major operators. Sent both Singapore rows within confirmed
business hours (~10:17 SGT): ESR Group (Philemon Foo) and ASE Singapore.

CRM now at 110 total (105 sent, 5 bounced, 4.5% hard-bounce rate -- no
new bounces today, but still over the 2% ceiling from the 3 bounces
2 days ago).

This is a real strategic inflection point, not a one-off slow day --
see conversation for the options being put to the owner (accept lower
volume, loosen the evidence bar, or expand scope to a new market).
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U109"/>
+  <dimension ref="A1:U111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8895,6 +8895,164 @@
       <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr"/>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>bd@aseglobal.com.sg</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Business Development</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ASE Singapore Pte Ltd</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://www.aseglobal.com.sg</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>web_research: https://www.digitimes.com/news/a20250519PD208/ase-singapore-testing-investment-siph.html — ASE is expanding and reinventing its Singapore chip-testing operations, investing in silicon photonics and co-packaged optics (CPO) test capability, positioning its Singapore site within Southeast Asia's AI data-center supply chain</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L110" t="n">
+        <v>1</v>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>1a0a801752096178</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>2026-09-16T02:17:36+00:00</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>2026-09-16T02:17:47+00:00</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R110" t="inlineStr"/>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr"/>
+      <c r="U110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>media@esr.com</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Philemon Foo</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Group Communications Manager, ESR</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ESR Group</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://www.esr.com</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>web_research: https://www.esr.com/news/esr-appoints-dalmar-sheikh-ceo-data-centres/ — ESR appointed Dalmar Sheikh as CEO of ESR Data Centres (effective 1 Sept 2026), based in Singapore, to lead the group's data centre platform, which carries a pipeline of more than 3.2GW across major Asia-Pacific markets amid rising hyperscaler and enterprise AI demand</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>1</v>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>1a0a8016ebbaec1e</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>2026-09-16T02:17:36+00:00</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>2026-09-16T02:17:47+00:00</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R111" t="inlineStr"/>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr"/>
+      <c r="U111" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct BDDC bounce: sent -> bounced (connection timeout, day 5 health check)
Gmail exhausted its retry window on sales@bd-dc.com (Bersama Digital
Data Centers) after two delay notices and a final 4.4.1 "recipient
server did not accept our requests to connect" on 2026-09-17 -- a
genuine hard failure, not a transient still in flight. Corrected in the
CRM. Hard-bounce rate now 6 bounced / 104 sent / 110 total = 5.455%,
over 2.7x the 2% ceiling.

No new sends today -- Indonesia and Singapore research both returned
zero audit-clean prospects for the third and second consecutive day
respectively. 71/71 tests pass.
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -6731,28 +6731,24 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>sent</t>
+          <t>bounced</t>
         </is>
       </c>
       <c r="L81" t="n">
         <v>1</v>
       </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>1a09d4f5a0396323</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>SMTP 4.4.1: The recipient server did not accept our requests to connect (bd-dc.com timed out on all MX hosts); Gmail gave up after retrying, final DSN Action: failed, Last-Attempt-Date Wed 16 Sep 2026 21:16:49 -0700</t>
+        </is>
+      </c>
       <c r="O81" t="inlineStr">
         <is>
           <t>2026-09-14T00:25:16+00:00</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>2026-09-14T00:27:10+00:00</t>
-        </is>
-      </c>
+      <c r="P81" t="inlineStr"/>
       <c r="Q81" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>

<commit_message>
Day 6 send: 1 real email (Gorilla Technology Group, Indonesia)
Sent within confirmed WIB business hours (16:26). Hand-humanized with
a fresh opener and a genuinely composed closer tied to the specific
September 2026 deployment timeline -- not picked verbatim from _CTAS,
per the 2026-09-18 fix. Subject line uses the new question-style
rotation, distinct shape from the recent "[Company]'s [noun]" pattern.

CRM now at 111 total (105 sent, 6 bounced). Singapore: 0 today, third
straight empty/near-empty day.
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U111"/>
+  <dimension ref="A1:U112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9049,6 +9049,83 @@
       <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr"/>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>sales@gorilla-technology.com</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Gorilla Technology Group</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://www.gorilla-technology.com</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/gorilla-technology-secures-25bn-gpuaas-contract-in-indonesia/ — Signed a transformational US$2.5B, 5-year AI GPUaaS compute contract anchored at NeutraDC's Batam, Indonesia data center; first phase (~1,000 NVIDIA B300 GPU servers) targets deployment in September 2026, a high-density GPU buildout requiring serious thermal management</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L112" t="n">
+        <v>1</v>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>1a0c34a3062b0171</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:26:42+00:00</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>2026-09-21T09:26:59+00:00</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R112" t="inlineStr"/>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr"/>
+      <c r="U112" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Day 8 send: 3 real emails (1 Indonesia, 2 Singapore) from yesterday's prep
Sent within confirmed business hours (09:08 WIB, 10:08 SGT). All three
hand-humanized using the burstiness/structural-variety technique from
2026-09-18's research fix -- three distinct sentence forms across the
batch (fact-first/two-short, implication-first/one-long,
short-punch-then-elaborate), fresh composed CTAs (not pulled from the
_CTAS pool verbatim), varied question-style subjects.

Wang Junhong (NUS IT, real Tier-1 upgrade), Laura Chen (GDS
International, new Jurong East hyperscale site), PT Bali Towerindo
Sentra Tbk (Balitower/Balifiber).

CRM now at 114 total (108 sent, 6 bounced).
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U112"/>
+  <dimension ref="A1:U115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9126,6 +9126,241 @@
       <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr"/>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>business@balifiber.id</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>PT Bali Towerindo Sentra Tbk (Balitower / Balifiber Data Center)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://www.balifiber.id</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>web_research: https://www.balifiber.id/home/bt_datacenter ; cross-checked via https://tiaonline.org/942-datacenter/pt-bali-towerindo-sentra-tbk-bali-tower-sentra-data-center-jl-batu-ceper-no-53-kebon-kelapa-gambir-jakarta-pusat-10120/ and https://www.idnfinancials.com/archive/45596/bali-towerindo-sentra-reinforce-data-centre-cctv-business — IDX-listed tower/infrastructure operator (BALI) runs Balitower/Balifiber Data Center in Jakarta Pusat, a TIA-942 Rated 3 certified facility that has expanded</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L113" t="n">
+        <v>1</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>1a0c6dfee1d86767</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:08:54+00:00</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:09:24+00:00</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R113" t="inlineStr"/>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr"/>
+      <c r="U113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ir@gds-services.com</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Laura Chen</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Investor Relations, GDS Holdings Limited</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>GDS International (GDS Holdings)</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://www.gds-services.com</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/gds-acquires-singapore-warehouse-plans-data-center-redevelopment/ — GDS International (CEO Jamie Khoo) acquired a S$112.8M / 39,978 sqm site at 21 Jalan Buroh, Jurong East, Singapore for a new hyperscale data center, part of an 80MW EDB/IMDA capacity award shared with Equinix, Microsoft and AirTrunk</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L114" t="n">
+        <v>1</v>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>1a0c6dfe66d4f732</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:08:54+00:00</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:09:24+00:00</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R114" t="inlineStr"/>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr"/>
+      <c r="U114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>junhong@nus.edu.sg</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Wang Junhong</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Senior Manager (HPC-AI), NUS Information Technology</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>NUS IT (High Performance Computing)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://nusit.nus.edu.sg/hpc/</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>web_research: https://nusit.nus.edu.sg/hpc/wang-jun-hong (cross-checked via independent WebSearch query returning the same address, per this session's WebFetch-egress-blocked fallback protocol) — Named Senior Manager for NUS's centralized HPC-AI computing infrastructure (multi-core clusters, GPU accelerators) supporting compute-intensive research workloads across NUS -- a facilities/technical-operations-tier contact, not the general IT helpdesk inbox already on file</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L115" t="n">
+        <v>1</v>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>1a0c6dfdf93c8b16</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:08:54+00:00</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>2026-09-22T02:09:24+00:00</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R115" t="inlineStr"/>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr"/>
+      <c r="U115" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct Balifiber bounce, bounce rate now 6.14% and trending up
business@balifiber.id hard-bounced within seconds of sending (550 5.1.1,
address rejected). This is the 7th bounce total, 3 of the last 4 real
sends. Bounce rate: 107 sent / 7 bounced / 114 total = 6.14%, up from
5.45% yesterday -- getting worse, not better, as the pool thins into
lower-quality generic inboxes. Business-hours compliance stays 100%
since the 2026-09-12 fix (66/66).

This is a real pattern now, not noise -- flagging plainly rather than
just logging another correction.
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -9163,28 +9163,24 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>sent</t>
+          <t>bounced</t>
         </is>
       </c>
       <c r="L113" t="n">
         <v>1</v>
       </c>
-      <c r="M113" t="inlineStr">
-        <is>
-          <t>1a0c6dfee1d86767</t>
-        </is>
-      </c>
-      <c r="N113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>550 5.1.1 &lt;business@balifiber.id&gt;: Recipient address rejected: balifiber.id (mailer-daemon, 2026-09-22)</t>
+        </is>
+      </c>
       <c r="O113" t="inlineStr">
         <is>
           <t>2026-09-22T02:08:54+00:00</t>
         </is>
       </c>
-      <c r="P113" t="inlineStr">
-        <is>
-          <t>2026-09-22T02:09:24+00:00</t>
-        </is>
-      </c>
+      <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>

<commit_message>
Day 11: send 5 audited prospects; fix signal-extraction delimiter bug
Sent live to all 5 already-audited unsent rows (2 Indonesia: UGM, ITS;
3 Singapore: Bridge Data Centres, JTC/Jacqueline Poh, Empyrion
Digital/Phoebe Ewe) via email-outreach-agent, each humanized before
sending, all confirmed within business hours (09:15 WIB / 10:15 SGT).

Also fixed a real bug the sending agent flagged: _extract_signal_from_source()
only recognized " — " (em dash) as the Source-field delimiter, so any
row using " -- " (double hyphen) silently fell back to a generic,
signal-less opener in the raw template even though a real verified
signal was present in the data (caught on the ITS row this run). Now
accepts both delimiters.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U115"/>
+  <dimension ref="A1:U120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9357,6 +9357,387 @@
       <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr"/>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ad_wibawa@its.ac.id</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Ir. Adhi Dharma Wibawa, S.T., M.T.</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Head (Kepala Pusat), Center of AI and Digital Technology (AIDT/KATD)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>ITS</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>web_research: https://www.its.ac.id/katd/en/prof-dr-ir-adhi-dharma-wibawa-s-t-m-t/ ; cross-checked via a second independently-worded WebSearch query confirming ad_wibawa@its.ac.id appears on the AIDT/KATD centers own webinar content pages (per WebFetch-egress-blocked fallback protocol) -- Head of the ITS center that itself operates the NVIDIA DGX-A100 AI supercomputer cited in the existing ITS prospects.csv row (https://www.its.ac.id/komputer/id/launching-nvidia-dgx-a100-artificial-intelligence-</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L116" t="n">
+        <v>1</v>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc0d60f76f22a</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:16:46+00:00</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:17:13+00:00</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R116" t="inlineStr"/>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr"/>
+      <c r="U116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>jacqueline_poh@jtc.gov.sg</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Jacqueline Poh</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>JTC Corporation</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>web_research: https://www.mingtiandi.com/real-estate/data-centres/singapore-plans-700mw-data-centre-park-on-jurong-island/ — JTC set aside 20 hectares on Jurong Island for Singapore's largest low-carbon Data Centre Park (up to 700MW); CEO Jacqueline Poh personally quoted on the project as JTC's bold step to build infrastructure for this new low-carbon data-centre hub</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L117" t="n">
+        <v>1</v>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc0d6c7aa1d75</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:16:46+00:00</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:17:13+00:00</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R117" t="inlineStr"/>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr"/>
+      <c r="U117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>mardhani@ugm.ac.id</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Dr. Mardhani Riasetiawan</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Head of Digital Transformation Bureau (Kepala Biro Transformasi Digital)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Universitas Gadjah Mada</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>web_research: https://ugm.ac.id/en/news/ugm-partners-with-nvidia-and-indosat-to-advance-ai-research/ ; cross-checked via https://acadstaff.ugm.ac.id/mardhaniriasetiawan and https://mardhani.staff.ugm.ac.id/ (per WebFetch-egress-blocked fallback protocol, two independently-worded WebSearch queries both returned mardhani@ugm.ac.id) — Coordinated the UGM Indosat NVIDIA AI Technology Center launch (NVIDIA DGX Station AI supercomputer at Faculty of Engineering/Faculty of Mathematics and Natural Scien</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L118" t="n">
+        <v>1</v>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc0d59d1eafe3</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:16:46+00:00</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:17:13+00:00</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R118" t="inlineStr"/>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr"/>
+      <c r="U118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>media@bridgedatacentres.com</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Media Enquiries</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Bridge Data Centres</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">web_research: https://www.datacenterdynamics.com/en/news/bridge-data-centres-plans-to-invest-23bn-4bn-in-singapores-digital-infrastructure/ — CEO Eric Fan stated Bridge Data Centres plans to invest up to S$5B (~US$3.9B) in Singapore AI infrastructure, with research programs and facilities tied to advanced power architectures, next-generation cooling systems, AI-enabled operations, and energy optimization for high-density computing (cross-checked via Bloomberg and Mingtiandi coverage of the same </t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L119" t="n">
+        <v>1</v>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc0d66a738f75</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:16:46+00:00</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:17:13+00:00</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R119" t="inlineStr"/>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr"/>
+      <c r="U119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>phoebe.ewe@empyriondigital.com</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Phoebe Ewe</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>VP, Marketing &amp; Communications</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Empyrion Digital</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>web_research: https://empyriondigital.com/quantum-safe-and-ai-ready-empyrion-digitals-singapore-hub-expands-local-footprint-with-over-s1-1-billion-investment/ — Empyrion Digital (Singapore-HQ'd) investing over S$1.1B to expand Singapore data-centre capacity for high-density AI/cloud workloads; SG1 facility targets PUE below 1.20 and Green Mark Platinum certification; Phoebe Ewe is the named press contact on the company's own Singapore and Taiwan groundbreaking release boilerplate</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L120" t="n">
+        <v>1</v>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc0d739efeb23</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:16:46+00:00</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:17:13+00:00</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R120" t="inlineStr"/>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr"/>
+      <c r="U120" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 11 health check (no new bounces)
123 total rows, 116 sent, 7 bounced (unchanged) - bounce rate down to
5.69% with today's 9 sends added to the denominator.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U120"/>
+  <dimension ref="A1:U124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9738,6 +9738,326 @@
       <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr"/>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>fariz@ui.ac.id</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Fariz Darari, S.Kom., M.Sc., Ph.D.</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Faculty in Charge, Tokopedia-UI AI Center of Excellence</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Universitas Indonesia - Fasilkom (Tokopedia-UI AI Center)</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>https://tokopedia-ai.cs.ui.ac.id</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>web_research: https://cs.ui.ac.id/personnel/fariz-darari/ ; cross-checked via a second independently-worded WebSearch query returning the same fariz@ui.ac.id address consistently (per this session's WebFetch-egress-blocked fallback protocol) — Faculty lead at the Tokopedia-UI AI Center of Excellence, Indonesia's first AI development center, built around an NVIDIA DGX-1 deep-learning supercomputer hosted at Fasilkom UI -- a named, domain-matched (ui.ac.id) technical contact for a company already</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L121" t="n">
+        <v>1</v>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc179ddc13238</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:10+00:00</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:17+00:00</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R121" t="inlineStr"/>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr"/>
+      <c r="U121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>info@worldvueribyond.com</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>General Enquiries</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>WorldVuer iByond (Quantum AI Data Center, Batam)</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>https://www.worldvueribyond.com</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>web_research: https://bkpm.go.id/id/info/siaran-pers/ri-siap-fasilitasi-investasi-data-center-ai-pertama-di-asia-senilai-rp6-t ; cross-checked via https://kepri.antaranews.com/berita/228541/bkpm-fasilitasi-investasi-pusat-data-ai-pertama-di-asia-senilai-rp6-triliun-di-batam and a second independently-worded WebSearch query confirming info@worldvueribyond.com on the company's own worldvueribyond.com site (per WebFetch-egress-blocked fallback protocol) — BKPM-facilitated US$400M (~Rp6 trillion) jo</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L122" t="n">
+        <v>1</v>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc17cb57f253f</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:10+00:00</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:29+00:00</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R122" t="inlineStr"/>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr"/>
+      <c r="U122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>msudarma@unud.ac.id</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Ir. Made Sudarma, MASc., IPU., ASEAN Eng.</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Head, Udayana Center of Excellence for Artificial Intelligence (UCEAI)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Universitas Udayana</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://uceai.unud.ac.id</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>web_research: https://udayananetworking.unud.ac.id/lecturer/credential/3002-made-sudarma ; cross-checked via a second independently-worded WebSearch query returning the same msudarma@unud.ac.id address (per WebFetch-egress-blocked fallback protocol) — Heads UCEAI, Udayana's dedicated AI research center focused on AI development/application for Bali and Eastern Indonesia (same center already cited as the technology-need signal for the existing generic humas@unud.ac.id row) -- a named, domain-matc</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L123" t="n">
+        <v>1</v>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc17b2788383b</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:10+00:00</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:23+00:00</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R123" t="inlineStr"/>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr"/>
+      <c r="U123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>sally.comollo@global.ntt</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Sally Comollo</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Director of Communications, NTT Global Data Centers</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>NTT Global Data Centers (Singapore)</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://services.global.ntt</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>web_research: https://services.global.ntt/en-us/services-and-products/global-data-centers/global-locations/asia-pacific/serangoon-data-center — NTT operates Serangoon Data Center (SG1) in Singapore, its first self-built/self-managed DC outside Japan, running an N+1 chilled-water cooling system; NTT Global Data Centers own AI-and-HPC-ready-data-centers page (services.global.ntt) describes actively deploying liquid cooling and direct-to-chip cold plates across its portfolio including Asia-Pacific</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L124" t="n">
+        <v>1</v>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>gmail:1a0cc17e133672d6</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:10+00:00</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>2026-09-23T02:28:34+00:00</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr"/>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr"/>
+      <c r="U124" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 12 send batch (no new bounces, no blank websites)
130 total rows, 123 sent, 7 bounced (unchanged). All 7 of today's sends
have a populated website field - yesterday's blank-website bug did not
recur (sending agent was explicitly told to pass it through this time).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U124"/>
+  <dimension ref="A1:U131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10078,6 +10078,553 @@
       <c r="T124" t="inlineStr"/>
       <c r="U124" t="inlineStr"/>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>college_central@ite.edu.sg</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>General Enquiries</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Institute of Technical Education (ITE) College Central - AiTE</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://www.ite.edu.sg</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>web_research: https://thetechrevolutionist.com/2022/01/ite-and-nvidia-launch-ai-workforce-readiness-programme.html</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L125" t="n">
+        <v>1</v>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f59380c75d</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr"/>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr"/>
+      <c r="U125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>humas@pajak.go.id</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Public Relations (Humas), Direktorat Jenderal Pajak</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Direktorat Jenderal Pajak (DJP) - Kementerian Keuangan RI</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://www.pajak.go.id</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>web_research: https://www.liputan6.com/tekno/read/8295162/bangun-coretax-hingga-pusat-data-ai-lg-cns-sabet-penghargaan-dari-djp-kemenkeu</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L126" t="n">
+        <v>1</v>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f3bd0a204d</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr"/>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr"/>
+      <c r="U126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>info@smplus.com</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>SM+ Data Centers (PT DSST Mas Gemilang / Sinar Mas)</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>https://smplus.com</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>web_research: https://w.media/sm-data-centers-kira-and-lg-sinar-mas-top-out-smx01-in-jakarta/</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L127" t="n">
+        <v>1</v>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f35364a40f</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr"/>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr"/>
+      <c r="U127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>media@singaporetech.edu.sg</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Media Relations</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Singapore Institute of Technology (SIT)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>https://www.singaporetech.edu.sg</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>web_research: https://www.singaporetech.edu.sg/news/sit-marks-opening-its-flagship-ai-centre-sit-punggol-campus-key-initiatives-and-partnerships-advance</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L128" t="n">
+        <v>1</v>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f3eecdf3b7</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q128" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr"/>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr"/>
+      <c r="U128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>nuhs_media@nuhs.edu.sg</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Media Relations</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>National University Health System (NUHS)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>https://www.nuhs.edu.sg</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>web_research: https://www.nuhs.edu.sg/about-nuhs/contact-us</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L129" t="n">
+        <v>1</v>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f44088ec51</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr"/>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr"/>
+      <c r="U129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>pohseng@nus.edu.sg</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Assoc Prof Lee Poh Seng</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Programme Director, Sustainable Tropical Data Centre Testbed (STDCT); Head, Dept of Mechanical Engineering, NUS</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>National University of Singapore (NUS) - Sustainable Tropical Data Centre Testbed</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>https://cde.nus.edu.sg/me/staff/lee-poh-seng/</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>web_research: https://news.nus.edu.sg/worlds-first-tropical-climate-data-centre-testbed/</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L130" t="n">
+        <v>1</v>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f4a13d159b</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr"/>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr"/>
+      <c r="U130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ygwen@ntu.edu.sg</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Prof Wen Yonggang</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Programme Co-Director, Sustainable Tropical Data Centre Testbed (STDCT); Professor, NTU</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Nanyang Technological University (NTU) - Sustainable Tropical Data Centre Testbed</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://personal.ntu.edu.sg/ygwen/</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>web_research: https://news.nus.edu.sg/worlds-first-tropical-climate-data-centre-testbed/</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L131" t="n">
+        <v>1</v>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>gmail:1a0d13f53f00af9b</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:30+00:00</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>2026-09-24T02:29:49+00:00</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R131" t="inlineStr"/>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr"/>
+      <c r="U131" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 13 send batch (no new bounces, no blank websites)
138 total rows, 131 sent, 7 bounced (unchanged).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U131"/>
+  <dimension ref="A1:U139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10625,6 +10625,642 @@
       <c r="T131" t="inlineStr"/>
       <c r="U131" t="inlineStr"/>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>audrey.lau.l.p@singhealth.com.sg</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Audrey Lau</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Group Chief Communications Officer</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>SingHealth (Singapore General Hospital Campus)</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>https://www.singhealth.com.sg</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>web_research: https://www.singhealth.com.sg/news/announcements/supercomputer-for-complex-health-research-at-new-centre</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L132" t="n">
+        <v>1</v>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>1a0d65fddfe6c101</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr"/>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr"/>
+      <c r="U132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>help-occ@rp.edu.sg</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Office of Corporate Communications</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Republic Polytechnic (RP) - AI Technology Centre (AITC)</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>https://www.rp.edu.sg</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>web_research: https://www.rp.edu.sg/about-us/contact-us/</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L133" t="n">
+        <v>1</v>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>1a0d65fe2e523eb5</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr"/>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr"/>
+      <c r="U133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ir@digitalcorereit.com</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Mabel Tan</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Director, Capital Markets &amp; Investor Relations</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Digital Core REIT</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>https://www.digitalcorereit.com</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>web_research: https://www.digitalcorereit.com/investor-relations/email-alerts-and-ir-contact/default.aspx</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L134" t="n">
+        <v>1</v>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>1a0d65fea7d8bcae</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr"/>
+      <c r="U134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ir@superx.sg</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Investor Relations</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>SuperX AI Technology Limited</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://www.superx.sg</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>web_research: https://www.prnewswire.com/news-releases/ai-compute-simplified-st-telemedia-global-data-centres-and-super-x-0cmut4phmwuj.html</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L135" t="n">
+        <v>1</v>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>1a0d65fefbbb0c20</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr"/>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr"/>
+      <c r="U135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>marketing@bitera-dc.com</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Tedy Harjanto</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Bitera Data Center (PT Mitra Informatika Gemilang)</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>https://www.bitera-dc.com/</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/bitera-data-center-in-jakarta-indonesia-launches-operations/</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L136" t="n">
+        <v>1</v>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>1a0d65fca086c963</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr"/>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr"/>
+      <c r="U136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>media@certisgroup.com</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Media Contact</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Certis Group</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>https://www.certisgroup.com</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>web_research: https://servers.asus.com/stories/Certis</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L137" t="n">
+        <v>1</v>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>1a0d65ff49a422a6</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr"/>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr"/>
+      <c r="U137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>sales@dtp.net.id</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Michael Alifen</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Director &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>DTP (PT Dwi Tunggal Putra)</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://www.dtp.net.id/</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>web_research: https://www.dtp.net.id/en/data-center-services/data-center</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L138" t="n">
+        <v>1</v>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>1a0d65fd53ad6410</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr"/>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr"/>
+      <c r="U138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>sales@mettadc.com</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Sukoco Halim</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>President Director &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>MettaDC (PT MettaDC Teknologi Indonesia)</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://mettadc.com/</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>web_research: https://www.theiconomics.com/market-expansion/proyek-pertama-resmi-beroperasi-mettadc-akan-terus-bangun-data-center-hingga-500-mw/</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L139" t="n">
+        <v>1</v>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>1a0d65fd1d7dced6</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:13+00:00</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>2026-09-25T02:23:32+00:00</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr"/>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr"/>
+      <c r="U139" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 14 send batch (no new bounces, no blank websites)
143 total rows, 136 sent, 7 bounced (unchanged).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U139"/>
+  <dimension ref="A1:U144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11261,6 +11261,403 @@
       <c r="T139" t="inlineStr"/>
       <c r="U139" t="inlineStr"/>
     </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>info@inti.co.id</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>PT INTI (Persero)</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://www.inti.co.id</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>web_research: https://www.inti.co.id/?p=13158 — State-owned telecom manufacturer PT INTI (Persero) is developing an AI GPU-based Data Center on its 8-hectare Bandung headquarters site (3,888 sqm operational facility), per its own site news and a May 2024 MoU with PT Jagat Bali Lestari to build and operate the facility, corroborated by a second independent report (i-portal.inti.co.id/post/4379/bandung-punya-ai-data-center) confirming the AI GPU data center is being developed there.</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L140" t="n">
+        <v>1</v>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>gmail:1a0e5d4b636224a8</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:25+00:00</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr"/>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr"/>
+      <c r="U140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>kee_yuan_ngiam@nuhs.edu.sg</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>A/Prof Ngiam Kee Yuan</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Group Chief Technology Officer &amp; Head, AI Office, NUHS</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>NUHS</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://www.nuhs.edu.sg</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>web_research: https://www.biospectrumasia.com/company-results/54/22939/singapores-nuhs-launches-first-ai-driven-supercomputer-to-empower-healthcare-projects.html ; contact confirmed via https://discovery.nuhs.edu.sg/2737-kee-yuan-ngiam and https://www.sgdi.gov.sg/ministries/moh/others/nuhs/departments/gito/Departments/aio — Leads NUHS's AI Office and the Prescience supercomputer initiative -- Singapore's third national supercomputer and first in healthcare, running multiple NVIDIA DGX A100 nodes for medical LLM training, built with NSCC -- a genuinely on-point named lead for the facility already cited as NUHS's technology-need signal</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L141" t="n">
+        <v>1</v>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>gmail:1a0e5d4bc6a7e193</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:25+00:00</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr"/>
+      <c r="U141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>media@ovhcloud.com</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Marie Vaillaud</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Communications and PR Manager</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>OVHcloud Singapore</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://www.ovhcloud.com/en-sg/</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/ovhcloud-launches-data-center-in-singapore/ ; press contact confirmed via corporate.ovhcloud.com newsroom boilerplate — OVHcloud launched SGP2, its second Singapore data center, billed as its most sustainable APAC facility, expanding Bare Metal/dedicated server capacity to meet regional AI and cloud demand</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L142" t="n">
+        <v>1</v>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>gmail:1a0e5d4c0d85fdf2</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:25+00:00</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr"/>
+      <c r="U142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>rickie.patani@nus.edu.sg</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Prof Rickie Patani</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Professor of Neuroscience &amp; Director, Neurobiology Programme, Life Sciences Institute, NUS Medicine</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>NUS Medicine</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://medicine.nus.edu.sg</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>web_research: https://medicine.nus.edu.sg/news/nus-medicine-dayone-and-cortical-labs-unveil-biological-data-center-prototype-in-singapore/ ; contact confirmed via https://www.nus.edu.sg/lsi/principal-investigators-3/prof-rickie-patani/ — NUS Medicine, DayOne Data Centers and Cortical Labs unveiled a Biological Data Centre prototype in Singapore (Aug 2026) -- 20 CL1 biological-computing units powered by 16 million living human neurons, requiring precise thermal/environmental control per rack; Prof Patani supervises the neuron cultures used in the deployment as Director of NUS LSI's Neurobiology Programme</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L143" t="n">
+        <v>1</v>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>gmail:1a0e5d4b9cc3375b</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:25+00:00</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr"/>
+      <c r="U143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>zhengkui.wang@singaporetech.edu.sg</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Daniel Zhengkui Wang</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Director, SIT x NVIDIA AI Centre (SNAIC) &amp; Associate Professor, Infocomm Technology Cluster</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Singapore Institute of Technology</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://www.singaporetech.edu.sg</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>web_research: https://www.singaporetech.edu.sg/news/sit-marks-opening-its-flagship-ai-centre-sit-punggol-campus-key-initiatives-and-partnerships-advance ; contact confirmed via https://www.singaporetech.edu.sg/directory/faculty/daniel-zhengkui-wang — Director of SIT's flagship SNAIC facility at Punggol Campus, a ~250 sqm AI centre built around an NVIDIA DGX H200 serving 50+ research engineers/students and 20+ industry partners -- a real, named lead for the same facility already cited as SIT's technology-need signal</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L144" t="n">
+        <v>1</v>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>gmail:1a0e5d4ba7fdb5f0</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:06+00:00</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>2026-09-28T02:25:25+00:00</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr"/>
+      <c r="U144" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 14 bounce correction (WorldVuer iByond)
143 total rows, 135 sent, 8 bounced (5.59%). WorldVuer iByond's Day 13
temporary delivery-delay notice (4.4.1 SMTP timeout, 45-hour retry
window) has now resolved to a hard failure - corrected from sent to
bounced by reporting-agent's health check, per the standing rule to
only mark bounced on a real mailer-daemon notification.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -9880,7 +9880,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>sent</t>
+          <t>bounced</t>
         </is>
       </c>
       <c r="L122" t="n">
@@ -9891,17 +9891,17 @@
           <t>gmail:1a0cc17cb57f253f</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr"/>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>4.4.1 The recipient server did not accept our requests to connect (timed out after 45h retry window); [worldvueribyond.com 2606:4700:3034::ac43:951d: timed out] [worldvueribyond.com 2606:4700:3032::6815:21c8: timed out] [worldvueribyond.com 172.67.149.29: timed out] [worldvueribyond.com 104.21.33.200: timed out]</t>
+        </is>
+      </c>
       <c r="O122" t="inlineStr">
         <is>
           <t>2026-09-23T02:28:10+00:00</t>
         </is>
       </c>
-      <c r="P122" t="inlineStr">
-        <is>
-          <t>2026-09-23T02:28:29+00:00</t>
-        </is>
-      </c>
+      <c r="P122" t="inlineStr"/>
       <c r="Q122" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>

<commit_message>
Re-export CRM after Day 16 send batch (no new bounces, no blank websites)
155 total rows, 147 sent, 8 bounced (unchanged).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U146"/>
+  <dimension ref="A1:U156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11812,6 +11812,796 @@
       <c r="T146" t="inlineStr"/>
       <c r="U146" t="inlineStr"/>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>allocare@allobank.com</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Allo Bank Indonesia</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://www.allobank.com</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>0822 0822 4110</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>080 4110 4110</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>web_research: https://tiaonline.org/942-datacenter/pt-allo-bank-indonesia-tbk-data-center-allo-bank/ ; contact confirmed via Allo Bank official verified account, e.g. https://x.com/AlloBankID/status/2011269529486442641 — Allo Bank separated its infrastructure from parent Bank Mega and launched its own dedicated, TIA Rated-3 certified data center in May 2024</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L147" t="n">
+        <v>1</v>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028608588884</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>ap.ask@global.ntt</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>NTT Indonesia (NTT Global Data Centers)</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://services.global.ntt</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>+65 6991 2020</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>web_research: https://services.global.ntt/en-us/services-and-products/global-data-centers/global-locations/asia-pacific/jakarta-2a-data-center ; contact confirmed via https://services.global.ntt/en-us/speak-to-our-experts and https://services.global.ntt/en-us/services-and-products/global-data-centers/global-locations/asia-pacific — Jakarta 2 Annex (JKT2A), NTT's third Indonesia facility, delivers 12MW of IT load purpose-built for high-density deployments supporting racks up to 40kW, opening early 2026</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L148" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028ba720fbc3</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr"/>
+      <c r="U148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>callcenter@dukcapil.kemendagri.go.id</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Ditjen Dukcapil, Kemendagri (Data Center Ampera)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://dukcapil.kemendagri.go.id</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>08118005373</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>1500537</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>web_research: https://nirmedia.co/dukcapil-hadapi-tantangan-2026-dengan-penguatan-digitalisasi-dan-integritas/ ; contact confirmed via Ditjen Dukcapil official verified account, e.g. https://x.com/dukcapil168/status/1691300522341617665 — Building a Tier 3 data center ('Data Center Ampera') at the IPDN campus on Jalan Ampera, Jakarta, as backbone infrastructure for national population-data digital services, alongside expanded biometric servers and storage capacity</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>gmail:1a0f02878d0e9351</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>contactus@bankbsi.co.id</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>I Wayan Pulantara</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>AI Strategy &amp; Innovation Department Head</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Bank Syariah Indonesia (BSI)</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://www.bankbsi.co.id</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>081584114040</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>14040 / +62 21 80639999</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>web_research: https://teknologi.bisnis.com/read/20260617/84/1981304/bsi-bris-targetkan-infrastruktur-ai-gateway-rampung-tahun-ini ; contact confirmed via BSI verified official account, e.g. https://x.com/bankbsi_id/status/1669650245427544065 — Building an internal 'AI Gateway' computing infrastructure targeted for completion in 2026 to support internal AI applications and prevent shadow AI use, per AI Strategy &amp; Innovation Department Head I Wayan Pulantara at the Indonesia Ethical AI Summit (June 2026)</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L150" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>gmail:1a0f02839627f518</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>info@idc.co.id</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>IDC Indonesia (PT Internetindo Data Centra Indonesia)</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://www.idc.co.id</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>+62 21 526-9988</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>web_research: https://www.idc.co.id/ — Indonesia's first carrier-neutral data center operator, now operating 6 facilities across Jakarta, Batam, Bandung, Surabaya and Makassar carrying over 95% of Indonesian internet traffic — Indonesia's first carrier-neutral data center operator, now operating 6 facilities across Jakarta, Batam, Bandung, Surabaya and Makassar carrying over 95% of Indonesian internet traffic</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028bc989ed33</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr"/>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr"/>
+      <c r="U151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>marketing@ag-it.com</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr"/>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Astragraphia Information Technology (AGIT)</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://www.ag-it.com</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>(021) 2924 1177</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>web_research: https://www.itworks.id/53011/lewat-anak-usaha-astra-graphia-berencana-perkuat-bisnis-data-center.html ; contact confirmed via https://www.ag-it.com/contact-us — Astra Graphia's IT subsidiary AGIT is expanding its data center business and partnering with HPE and Equinix to build AI-based private cloud infrastructure for the Indonesian market</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L152" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028a5a72f66f</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr"/>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr"/>
+      <c r="U152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>marketing@nongsadigital.com</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Nongsa Digital Park (Citramas Group)</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://nongsadigital.com</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>+62 778 7100 673</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>web_research: https://nongsadigital.com/dc-hub-ndp/8-data-centre-infrastructure-nongsa-digital-park ; contact confirmed via https://nongsadigital.com/contact-us/ — NDP1 facility at Nongsa Digital Park (Batam) is designed for high-density enterprise, cloud, and AI workloads, with planned IT capacity of 120MW, hosting multiple data center operators (BW Digital, DayOne, Golden Digital Gateway, Racks Central) on its own park infrastructure</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>gmail:1a0f02876c4ba0c6</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>marketingicp@iconpln.co.id</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>PLN Icon Plus (PT Indonesia Comnets Plus)</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://www.plniconplus.co.id</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>web_research: https://listrikindonesia.com/detail/14093/energi-bersih-pln-icon-plus-siap-dukung-proyek-data-center-indonesia ; contact confirmed via the company's own site, https://lights.iconpln.co.id/article/37 (iconpln.co.id and plniconplus.co.id are the same company under its PLN Icon Plus rebrand, per https://iconews.iconpln.co.id/rebranding-pln-icon-plus-setting-tone-from-the-top/) — PLN Icon Plus (ICON+), PLN's telecom/data center subsidiary, states its commitment to supporting green data center development in Indonesia and operates its own DC2 data center facility amid rising AI-driven power and cooling demand</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028a241d929f</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>noc@napinfo.co.id</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Matrix NAP Info (PT NAP Info Lintas Nusa)</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://www.napinfo.co.id</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>1-500-787 / +62 21 3970 1787</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>web_research: https://napinfo.co.id/highlights/article/id/matrix-nap-info-jalin-kerja-sama-strategis-dengan-digital-realty-bersama-untuk-perkuat-ekosistem-infrastruktur-digital-nasional ; contact confirmed via https://www.napinfo.co.id/contact-us — Matrix NAP Info operates its own Matrix Data Center and struck a strategic partnership with Digital Realty Bersama to strengthen Jakarta data center interconnection for AI/cloud growth</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L155" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028620d291fb</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>support@lintasarta.co.id</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Lintasarta (PT Aplikanusa Lintasarta)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>https://www.lintasarta.net</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>08561114052</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>14052 / +62 21 80669499</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>web_research: https://freehire.me/jobs/cloud-data-center-engineer-gpu-openstack-lintasarta-qdsgh4bu and https://freehire.me/jobs/data-center-engineer-l2-lintasarta-qkksv7zy ; contact confirmed via https://www.lintasarta.net/en/contact-us/ — Actively hiring multiple onsite 24x7 Data Center Engineers (L1/L2/L3) for a large-scale GPU cloud built on rack-scale NVIDIA GB200 NVL72, with explicit responsibility for liquid-cooling systems (CDU and secondary loop) operation, monitoring and anomaly handling, alongside its NVIDIA-powered GPU Merdeka sovereign AI GPUaaS cloud already launched</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L156" t="n">
+        <v>1</v>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>gmail:1a0f028365b6c54f</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:32:36+00:00</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>2026-09-30T02:33:22+00:00</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr"/>
+      <c r="U156" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-export CRM after Day 17 Singapore send batch (no new bounces)
172 total rows, 164 sent, 8 bounced (unchanged). Indonesia batch for
today still in progress.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U156"/>
+  <dimension ref="A1:U173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12602,6 +12602,1379 @@
       <c r="T156" t="inlineStr"/>
       <c r="U156" t="inlineStr"/>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>christina.koh@sttelemediagdc.com</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Christina Koh</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Head, Group Marketing and Communications</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>ST Telemedia Global Data Centres</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>https://www.sttelemediagdc.com</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>web_research: https://www.sttelemediagdc.com/newsroom/st-telemedia-global-data-centres-announces-new-executive-appointments — STT GDC operates multiple Singapore data centre campuses and is developing the FutureGrid HVDC-AI testbed; Christina Koh is named alongside Chow Yi as the company's own media contact across its newsroom press releases.</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L157" t="n">
+        <v>1</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547310677735</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr"/>
+      <c r="U157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>contactus@synapxe.sg</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>General Enquiries</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Synapxe</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://www.synapxe.sg</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>web_research: https://www.synapxe.sg/healthtech/cloud/h-cloud — Synapxe, Singapore's national HealthTech agency, built H-Cloud to rationalise and consolidate local hospital data centres into a modernised, nation-wide private cloud serving all public hospitals, specialty centres, polyclinics and nursing homes.</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L158" t="n">
+        <v>1</v>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472d8f8548c</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr"/>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr"/>
+      <c r="U158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>corpcomms@ocbc.com</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr"/>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Group Brand and Communications</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>OCBC Bank</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://www.ocbc.com</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/singapores-ocbc-bank-to-introduce-rack-based-data-center-cooling/ — OCBC operates its own S$240M purpose-built data center in Singapore (first purpose-built DC owned by a Singapore bank) and is implementing a rack-based cooling system to cut emissions by 400+ tons/year; separately hiring a Data Centre Facilities Engineer and a Lead, Data Centre Facilities Management (AVP/VP) for the Loyang facility.</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L159" t="n">
+        <v>1</v>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5471f98cfb7a</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr"/>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr"/>
+      <c r="U159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>investor.relations@keppeldcreit.com</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr"/>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Investor Relations</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Keppel DC REIT</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://www.keppeldcreit.com</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>web_research: https://www.keppeldcreit.com/en/investor-relations/ir-contact/ — Keppel DC REIT is participating in the Keppel DC Singapore 9 build at the AI-ready Genting Lane campus (construction start mid-2026, 19MW), alongside Keppel Data Centre Funds II and III.</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L160" t="n">
+        <v>1</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54728c833da5</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr"/>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr"/>
+      <c r="U160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ir_industrial@mapletree.com.sg</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Cheng Mui Lian</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Investor Relations and Sustainability</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Mapletree Industrial Trust</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://www.mapletreeindustrialtrust.com</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>web_research: https://www.mapletreeindustrialtrust.com/about-us/ — Mapletree Industrial Trust's data-centre portfolio is roughly 57% of its S$8.3B total AUM, including the purpose-built 7 Tai Seng Drive facility (fully leased to Equinix Singapore) and the Sunview Drive data centre in Singapore, plus 13 data centres held via JV with Mapletree Investments in North America.</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L161" t="n">
+        <v>1</v>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54724a989642</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr"/>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr"/>
+      <c r="U161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>lauren.crystal@smc.co</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Lauren Crystal</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Head of Communications</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Sustainable Metal Cloud (SMC)</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://smc.co</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/singapores-sustainable-metal-cloud-outlines-global-expansion-plans/ — Singapore-founded and HQ'd SMC runs fully immersion-cooled NVIDIA GPU clusters (SIN01/SIN02 availability zones at STT GDC) for AI training/inference, achieving a PUE of 1.03 via its HyperCube immersion-cooling technology.</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L162" t="n">
+        <v>1</v>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472318d99a1</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr"/>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr"/>
+      <c r="U162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>luana.low@gf.com</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Luana Low</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Deputy Director, Corporate Communications (Public Relations, Singapore)</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>GlobalFoundries Singapore</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://gf.com</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>web_research: https://www.edb.gov.sg/en/about-edb/media-releases-publications/globalfoundries-opens-us4-billion-expansion-facility-in-singapore.html — GlobalFoundries officially opened a US$4B expansion fab in Singapore (23,000 sqm), its most advanced Singapore semiconductor facility to date, raising overall Singapore capacity to ~1.5M 300mm wafers/year.</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L163" t="n">
+        <v>1</v>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547267649121</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr"/>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr"/>
+      <c r="U163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>nola.pocock@colt.net</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Nola Pocock</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>VP, Global Communications (Colt Group)</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Colt Data Centre Services Singapore</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://www.coltdatacentres.net</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>web_research: https://www.colt.net/resources/insights/connectivity-for-mc-digital-realty-data-centre — Colt operates a Singapore data center at 29A International Business Park Road; Colt Group's own Global Communications lead (covering both Colt Technology Services and Colt Data Centre Services announcements) is Nola Pocock, consistently listed as press contact on colt.net data-centre-related releases.</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L164" t="n">
+        <v>1</v>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472e0be35ce</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr"/>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr"/>
+      <c r="U164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>tanya.netto@oracle.com</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Tanya Netto</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Communications &amp; PR Lead, ASEAN</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure Singapore</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/sg/</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>web_research: https://blogs.oracle.com/cloud-infrastructure/oracle-opens-second-cloud-region-in-singapore — Oracle opened a second Oracle Cloud Region in Singapore to meet rapidly growing AI/cloud demand, enabling customers to migrate mission-critical AI workloads.</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L165" t="n">
+        <v>1</v>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5472bfb7b7c4</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:14+00:00</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:45+00:00</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R165" t="inlineStr"/>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr"/>
+      <c r="U165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>ai.center@binus.edu</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Prof. Bens Pardamean</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Director, Artificial Intelligence R&amp;D Center (AIRDC)</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>BINUS University (AI R&amp;D Center)</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://research.binus.ac.id/airdc/</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>+62.21 530 0244</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>web_research: https://research.binus.ac.id/airdc/ ; https://binus.ac.id/2019/04/binus-dirikan-pusat-riset-artificial-intelligence/ — BINUS University AI R&amp;D Center (AIRDC), founded via NVIDIA-BINUS collaboration, operates a GPU cluster for AI research and industry collaboration, directed by Prof. Bens Pardamean</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L166" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475eb87633c</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr"/>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr"/>
+      <c r="U166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>corsec@pancaanugrahwisesa.com</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr"/>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Corporate Secretary</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>PT NexAI Digital Infrastruktur Tbk (MGLV, formerly PT Panca Anugrah Wisesa Tbk)</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>http://pancaanugrahwisesa.com</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>+62 21 718 0349</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>web_research: https://harianenergi.com/detail/1440376/dapat-restu-rupslb-nexai-mantap-garap-bisnis-ai-data-center ; https://bisnisinsight.com/detail/921750/nexai-mglv-resmi-masuk-bisnis-ai-data-center-usai-restu-rupslb — IDX-listed PT NexAI Digital Infrastruktur Tbk (MGLV) received shareholder approval (RUPSLB, July 2026) to formally pivot its core business from furniture/household equipment to AI-based data center infrastructure</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L167" t="n">
+        <v>1</v>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475ddf337f9</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr"/>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr"/>
+      <c r="U167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>info@edgnex.com</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr"/>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>DAMAC Digital (EDGNEX Cikarang AI Campus)</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://www.edgnex.com</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>+971 4 373 2 373</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>web_research: https://www.edgnex.com/contact/ ; https://www.idnfinancials.com/news/56071/dubais-damac-digital-to-build-usd-2-3-billion-data-centre-in-cikarang — DAMAC Digital (EDGNEX) is building a $2.3B AI data center in Greenland International Industrial Center, Pasirranji, Bekasi (JKT02/Cikarang AI Campus), designed for high-density AI racks with a projected capacity exceeding 144MW, first phase slated for Q3 2026 completion</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L168" t="n">
+        <v>1</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54759960550c</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R168" t="inlineStr"/>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr"/>
+      <c r="U168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>infodgx@gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Prof. Dr. Detty Purnamasari</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Head, AI and Robotics Development Team (DGX Development Team)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Universitas Gunadarma</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://www.hpc-hub.gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>+628-1212-9955-61</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>web_research: https://www.praktikum-hpc.gunadarma.ac.id/kontak/tim-pengembangan-dgx ; https://www.hpc-hub.gunadarma.ac.id/kontak — Prof. Dr. Detty Purnamasari heads the DGX Development Team overseeing Gunadarma University NVIDIA DGX-1 and DGX A100 supercomputers at its dedicated HPC/DGX hub for AI and data-intensive research</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54761cbada73</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:58+00:00</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr"/>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr"/>
+      <c r="U169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>inquiry@indokeppeldc.com</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr"/>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>IndoData Data Center (Salim Group, formerly IndoKeppel Data Centres)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>https://indokeppeldc.com</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>+622139520140</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/keppel-salim-group-launch-data-center-in-bogor-indonesia/ ; https://w.media/indokeppel-sees-significant-data-center-opportunities-in-indonesia/ — IndoKeppel Data Centre 1 (IKDC1) in Bogor, a Salim Group/Keppel JV (Salim Group took full ownership in Dec 2025 and relaunched as IndoData Data Center), is a 7-hectare campus planned for 50MW+ of IT power across 3 phases, featuring N+1 water-cooled chillers and dual water supply, with a stated strategic focus on AI and hyperscale computing; IndoData has up to 500MW of power capacity secured under contract with PLN</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475268bea7a</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr"/>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr"/>
+      <c r="U170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>inquiry@lgsinarmas.com</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr"/>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>General/Corporate Contact</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>LG Sinar Mas Technology Solutions (LG CNS / SM+ JV)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://www.lgsinarmas.com</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>+62-21-31990258</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>web_research: https://www.sinarmas.com/blog/?p=4168 ; https://www.lgsinarmas.com/ — LG Sinar Mas, a joint venture between South Korean DC services provider LG CNS and Sinar Mas-backed PT SMPlus Digital Investment (SM+), is developing a US$300M AI-based data center on a 44,195 sqm facility in Menteng Atas, Setiabudi, Jakarta, scheduled to begin operations in H2 2026</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L171" t="n">
+        <v>1</v>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>gmail:1a0f54756301e30b</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr"/>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr"/>
+      <c r="U171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>sales@dhs-dc.com</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Stanley Go</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Digital Hyperspace Indonesia (DHI)</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://dh-indonesia.com</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>web_research: https://dh-indonesia.com/contact/ ; https://dh-indonesia.com/about/ — PT Digital Hyperspace Indonesia operates DHI, a Tier III hyperscale data center in Pasirranji, Central Cikarang, Bekasi Regency, West Java, with an initial 20MW IT load (1,200,000 SF purpose-built facility), financed by the GTC Fund and co-investors; Operations Manager Stanley Go is ASHRAE BCxP-certified</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L172" t="n">
+        <v>1</v>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>gmail:1a0f547554b25881</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr"/>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr"/>
+      <c r="U172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>selena.sheikh@princetondg.com</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Selena Sheikh</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Corporate Communications Associate Director, Public Relations</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Princeton Digital Group (PDG) Indonesia</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://princetondg.com</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>web_research: https://princetondg.com/newsroom/princeton-digital-group-launches-its-22mw-hyperscale-data-center-in-greater-jakarta-2/ — PDG operates JC1 (6MW) and JC2 (22MW hyperscale, launched) data centers in Cibitung, Greater Jakarta, and agreed to acquire a 70%% stake in XL Axiata Indonesian data centers (5 sites) with US$100M growth capital committed to expand capacity</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="L173" t="n">
+        <v>1</v>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>gmail:1a0f5475a8ba596c</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:30+00:00</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>2026-10-01T02:24:57+00:00</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr"/>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr"/>
+      <c r="U173" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct LG Sinar Mas bounce (550 5.4.1 rejection), rate now 5.23%
LG Sinar Mas's Day 17 send (inquiry@lgsinarmas.com) bounced hard
5 minutes after sending - Microsoft/Outlook EXO rejected the address.
Corrected sent -> bounced, message_id preserved as proof-of-send.
9/172 = 5.23%, still above the 2% ceiling, now worse than yesterday's
4.65% (which itself hadn't caught this bounce yet).

No new sends happened today - the planned 11-email batch was blocked
at the permission layer (Gmail drafts only, not sent); this commit is
solely the bounce correction to an existing Day 17 row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -13777,7 +13777,7 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>sent</t>
+          <t>bounced</t>
         </is>
       </c>
       <c r="L171" t="n">
@@ -13788,17 +13788,17 @@
           <t>gmail:1a0f54756301e30b</t>
         </is>
       </c>
-      <c r="N171" t="inlineStr"/>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>550 5.4.1 Recipient address rejected: Access denied. (lgsinarmas-com.mail.protection.outlook.com)</t>
+        </is>
+      </c>
       <c r="O171" t="inlineStr">
         <is>
           <t>2026-10-01T02:24:30+00:00</t>
         </is>
       </c>
-      <c r="P171" t="inlineStr">
-        <is>
-          <t>2026-10-01T02:24:57+00:00</t>
-        </is>
-      </c>
+      <c r="P171" t="inlineStr"/>
       <c r="Q171" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>